<commit_message>
fix: SaveDataManager 데이타 싱크 로직 보완.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/PurchaseTable.xlsx
+++ b/input/Domains/Game/PurchaseTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D223F0DF-19E1-3E43-A446-5016C47805D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FCE3646-1F07-C14E-BCEE-38C5232D7CCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1420" yWindow="500" windowWidth="36980" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39820" yWindow="-1840" windowWidth="36980" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PRODUCT" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="33">
   <si>
     <t>internalProductId</t>
   </si>
@@ -70,17 +70,10 @@
     <t>Google Play SKU</t>
   </si>
   <si>
-    <t>Subscription</t>
-  </si>
-  <si>
     <t>com.devian.framework.product.noads_month</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>com.devian.framework.product.noads_subscription</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Rental</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -101,31 +94,46 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>chest_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>chest_002</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>chest_003</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>com.devian.framework.product.chest_003</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SeasonPass</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>pass_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reward_pass_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reward_chest_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>com.devian.framework.product.pass_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>noads_month</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>noads_subscription</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>chest_001</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>chest_002</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>chest_003</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>com.devian.framework.product.chest_003</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>reward_001</t>
+  </si>
+  <si>
+    <t>reward_noads_month</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -514,6 +522,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
     <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="43.42578125" bestFit="1" customWidth="1"/>
   </cols>
@@ -577,7 +587,7 @@
         <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s">
         <v>13</v>
@@ -591,88 +601,94 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
       </c>
       <c r="G6" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:G3 B6:D6 B5 F5 F6 D5 A4:B4 D4:G4" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:G3 F5 D5 A4:B4 D4:G4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: PurchaseManager 구매 버그 수정.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/PurchaseTable.xlsx
+++ b/input/Domains/Game/PurchaseTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FCE3646-1F07-C14E-BCEE-38C5232D7CCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F910F8-09D1-364D-86A3-C29BAFAFC4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39820" yWindow="-1840" windowWidth="36980" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3320" yWindow="500" windowWidth="36980" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PRODUCT" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
refactor: enum 이름 수정 및 input 파일 정리.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/PurchaseTable.xlsx
+++ b/input/Domains/Game/PurchaseTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F910F8-09D1-364D-86A3-C29BAFAFC4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC7C6F3D-8224-8C44-8834-A0374AD1A038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3320" yWindow="500" windowWidth="36980" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1420" yWindow="500" windowWidth="36980" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PRODUCT" sheetId="1" r:id="rId1"/>
@@ -46,9 +46,6 @@
     <t>string</t>
   </si>
   <si>
-    <t>ProductKind</t>
-  </si>
-  <si>
     <t>bool</t>
   </si>
   <si>
@@ -74,22 +71,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Rental</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>상품 타입 (Consumable/Rental/Subscription/SeasonPass)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>com.devian.framework.product.chest_001</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Consumable</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>com.devian.framework.product.chest_002</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -110,10 +95,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>SeasonPass</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>pass_001</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -134,6 +115,26 @@
   </si>
   <si>
     <t>reward_noads_month</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PRODUCT_KIND</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SEASON_PASS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CONSUMABLE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RENTAL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>상품 타입 (CONSUMABLE / RENTAL / SUBSCRIPTION / SEASON_PASS)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -559,13 +560,13 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
@@ -576,119 +577,119 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>13</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>14</v>
-      </c>
-      <c r="G4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
         <v>31</v>
-      </c>
-      <c r="B5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
         <v>24</v>
       </c>
-      <c r="B9" t="s">
-        <v>29</v>
-      </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:G3 F5 D5 A4:B4 D4:G4" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:G1 F5 D5 A4:B4 D4:G4 A3:G3 A2:B2 D2:G2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>